<commit_message>
Améliore le format des fiches navette et régénère les situations
- Bandeau vert "RenovBat Bureau d'Etude Bâtiment" sous le titre FICHE NAVETTE
- Supprime la ligne MOE/RenovBat devenue redondante
- Ajoute ligne Signataire J. Pons dans le bon de paiement
- Régénère les 3 fiches Excel et les fichiers de synthèse

https://claude.ai/code/session_01WPF94fYvsuR5JRX5sV8Vmx
</commit_message>
<xml_diff>
--- a/data/navettes_et_bons/lot01_Isolation_Thermique_PLAT001.xlsx
+++ b/data/navettes_et_bons/lot01_Isolation_Thermique_PLAT001.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00 &quot;EUR&quot;"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,18 +33,27 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="001E8449"/>
     </font>
     <font>
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E8449"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -59,12 +68,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -444,15 +456,10 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>MOE</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>RenovBat</t>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>RenovBat Bureau d'Etude Bâtiment</t>
         </is>
       </c>
     </row>
@@ -522,7 +529,7 @@
           <t>Montant HT</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="3" t="n">
         <v>10416.67</v>
       </c>
     </row>
@@ -532,7 +539,7 @@
           <t>TVA (20%)</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" s="3" t="n">
         <v>2083.33</v>
       </c>
     </row>
@@ -542,12 +549,12 @@
           <t>Montant TTC</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" s="3" t="n">
         <v>12500</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>✓ FACTURE APPROUVÉE</t>
         </is>
@@ -590,7 +597,7 @@
           <t>Budget total du lot HT</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n">
+      <c r="B21" s="3" t="n">
         <v>20000</v>
       </c>
     </row>
@@ -600,7 +607,7 @@
           <t>Budget total du lot TTC</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n">
+      <c r="B22" s="3" t="n">
         <v>24000</v>
       </c>
     </row>
@@ -610,7 +617,7 @@
           <t>Situations précédentes TTC</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n">
+      <c r="B24" s="3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -620,7 +627,7 @@
           <t>Présente situation HT</t>
         </is>
       </c>
-      <c r="B25" s="2" t="n">
+      <c r="B25" s="3" t="n">
         <v>10416.67</v>
       </c>
     </row>
@@ -630,7 +637,7 @@
           <t>Présente situation TVA</t>
         </is>
       </c>
-      <c r="B26" s="2" t="n">
+      <c r="B26" s="3" t="n">
         <v>2083.33</v>
       </c>
     </row>
@@ -640,7 +647,7 @@
           <t>Présente situation TTC</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n">
+      <c r="B27" s="3" t="n">
         <v>12500</v>
       </c>
     </row>
@@ -650,7 +657,7 @@
           <t>Nouveau cumul TTC</t>
         </is>
       </c>
-      <c r="B29" s="4" t="n">
+      <c r="B29" s="5" t="n">
         <v>12500</v>
       </c>
     </row>
@@ -660,7 +667,7 @@
           <t>Reste à régler TTC</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n">
+      <c r="B30" s="3" t="n">
         <v>11500</v>
       </c>
     </row>
@@ -691,18 +698,31 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>Signataire</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>J. Pons</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>À destination de</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>IMMOSOCIAL_69 (MOA)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A19:B19"/>
   </mergeCells>

</xml_diff>

<commit_message>
En-tête titulaire + bandeau vert BON DE PAIEMENT dans les fiches navette
- En-tête 4 colonnes (ENTREPRISE, lot, sit n°, fiche navette n°) en haut
  de chaque feuille, avec nom, adresse et intitulé du lot
- Bandeau vert "RenovBat Bureau d'Etude Bâtiment" ajouté sous BON DE PAIEMENT
- Références cellules mises à jour : B16 (TTC), A18 (statut approbation)
- process_situations.py : passe lot_num et adresse_prestataire au payload
- Résultats /situations régénérés

https://claude.ai/code/session_01WPF94fYvsuR5JRX5sV8Vmx
</commit_message>
<xml_diff>
--- a/data/navettes_et_bons/lot01_Isolation_Thermique_PLAT001.xlsx
+++ b/data/navettes_et_bons/lot01_Isolation_Thermique_PLAT001.xlsx
@@ -29,6 +29,9 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
       <sz val="13"/>
     </font>
     <font>
@@ -38,9 +41,6 @@
     <font>
       <b val="1"/>
       <color rgb="001E8449"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -56,7 +56,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -64,19 +64,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -442,289 +451,342 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>ENTREPRISE</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>sit n°</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>fiche navette n°</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Platr'O'Matic SARL</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>lot1 : Isolation thermique</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>42 rue du Crepissage - 75011 Paris</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
           <t>FICHE NAVETTE — PROJET renovation_2026</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>RenovBat Bureau d'Etude Bâtiment</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>MOA</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>IMMOSOCIAL_69</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Référence facture</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>FAC-2026-001</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Date de la facture</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>15 mars 2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Émetteur</t>
+          <t>MOA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Platr'O'Matic SARL</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Lot concerné</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>isolation_thermique</t>
+          <t>IMMOSOCIAL_69</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Montant HT</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>10416.67</v>
+          <t>Référence facture</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>FAC-2026-001</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TVA (20%)</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n">
-        <v>2083.33</v>
+          <t>Date de la facture</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>15 mars 2026</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Montant TTC</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n">
-        <v>12500</v>
+          <t>Émetteur</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Platr'O'Matic SARL</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Lot concerné</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>isolation_thermique</t>
+        </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>✓ FACTURE APPROUVÉE</t>
-        </is>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Montant HT</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>10416.67</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Date d'approbation</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>26/04/2026</t>
-        </is>
+          <t>TVA (20%)</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>2083.33</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>Montant TTC</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>12500</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>✓ FACTURE APPROUVÉE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Date d'approbation</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>Approuvé par</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>RenovBat</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>BON DE PAIEMENT — PROJET renovation_2026</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Budget total du lot HT</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="n">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Budget total du lot TTC</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="n">
-        <v>24000</v>
-      </c>
-    </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Situations précédentes TTC</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Présente situation HT</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="n">
-        <v>10416.67</v>
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>RenovBat Bureau d'Etude Bâtiment</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Présente situation TVA</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="n">
-        <v>2083.33</v>
+          <t>Budget total du lot HT</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="n">
+        <v>20000</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Présente situation TTC</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="n">
-        <v>12500</v>
+          <t>Budget total du lot TTC</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="n">
+        <v>24000</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Nouveau cumul TTC</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="n">
-        <v>12500</v>
+          <t>Situations précédentes TTC</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Reste à régler TTC</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="n">
-        <v>11500</v>
+          <t>Présente situation HT</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="n">
+        <v>10416.67</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Présente situation TVA</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="n">
+        <v>2083.33</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Date d'émission</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>26/04/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Établi par</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>RenovBat (MOE)</t>
-        </is>
+          <t>Présente situation TTC</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="n">
+        <v>12500</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Signataire</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>J. Pons</t>
-        </is>
+          <t>Nouveau cumul TTC</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="n">
+        <v>12500</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>Reste à régler TTC</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n">
+        <v>11500</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Date d'émission</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Établi par</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>RenovBat (MOE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Signataire</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>J. Pons</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>À destination de</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>IMMOSOCIAL_69 (MOA)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A19:B19"/>
+  <mergeCells count="5">
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A6:B6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>